<commit_message>
Fix plan, value sanity checks, duplicate detection, remembered paths
- Long sheet: LSL / Target / USL right after Unit_of_Measurement; Source_File
  and Open_File at the end.
- Fix plan: unambiguous folder repairs as a Fix_Plan sheet and a reviewable
  script; the converter never changes source folders itself.
- Sanity checks: Min/Mean/Max order, negative values, values far off the
  median of their block. Report only.
- Duplicate detection: identical workbook content in two places.
- App remembers the last folder and limits path.
- Stress project regenerated with physically ordered values and cases for the
  new checks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/Orion_Stress_Demo/PN-ALPHA-01/30101/BU 03/HRM/post FET_HRM-2031-0152/Panel-28/BACK/2031-03-01_08-00-00_ENG_Orion_Stress_Demo_BU03_Back_Summary.xlsx
+++ b/test_data/Orion_Stress_Demo/PN-ALPHA-01/30101/BU 03/HRM/post FET_HRM-2031-0152/Panel-28/BACK/2031-03-01_08-00-00_ENG_Orion_Stress_Demo_BU03_Back_Summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,26 +456,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pad 1</t>
+          <t>Pad Pos 1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>16.73274</v>
+        <v>16.89673</v>
       </c>
       <c r="D2" t="n">
-        <v>16.16827</v>
+        <v>16.49471</v>
       </c>
       <c r="E2" t="n">
-        <v>16.63397</v>
+        <v>16.73425</v>
       </c>
       <c r="F2" t="n">
-        <v>42.87933</v>
+        <v>41.96717</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05088</v>
+        <v>0.05178</v>
       </c>
       <c r="H2" t="n">
-        <v>1.86424</v>
+        <v>1.84251</v>
       </c>
     </row>
     <row r="3">
@@ -485,22 +485,22 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>16.70596</v>
+        <v>17.31653</v>
       </c>
       <c r="D3" t="n">
-        <v>16.54128</v>
+        <v>16.58718</v>
       </c>
       <c r="E3" t="n">
-        <v>16.94439</v>
+        <v>17.22145</v>
       </c>
       <c r="F3" t="n">
-        <v>42.76294</v>
+        <v>42.57334</v>
       </c>
       <c r="G3" t="n">
-        <v>0.05056</v>
+        <v>0.05027</v>
       </c>
       <c r="H3" t="n">
-        <v>1.80786</v>
+        <v>1.84047</v>
       </c>
     </row>
     <row r="4">
@@ -510,22 +510,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>16.90271</v>
+        <v>17.03701</v>
       </c>
       <c r="D4" t="n">
-        <v>16.68035</v>
+        <v>16.53639</v>
       </c>
       <c r="E4" t="n">
-        <v>16.55064</v>
+        <v>16.57017</v>
       </c>
       <c r="F4" t="n">
-        <v>42.77939</v>
+        <v>42.60183</v>
       </c>
       <c r="G4" t="n">
-        <v>0.05052</v>
+        <v>0.05126</v>
       </c>
       <c r="H4" t="n">
-        <v>1.83154</v>
+        <v>1.85419</v>
       </c>
     </row>
     <row r="5">
@@ -535,22 +535,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>17.0552</v>
+        <v>17.13978</v>
       </c>
       <c r="D5" t="n">
-        <v>16.55235</v>
+        <v>16.64321</v>
       </c>
       <c r="E5" t="n">
-        <v>16.81724</v>
+        <v>16.7137</v>
       </c>
       <c r="F5" t="n">
-        <v>42.97658</v>
+        <v>42.6672</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0503</v>
+        <v>0.05166</v>
       </c>
       <c r="H5" t="n">
-        <v>1.80459</v>
+        <v>1.78085</v>
       </c>
     </row>
     <row r="6">
@@ -560,22 +560,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>17.07742</v>
+        <v>16.93295</v>
       </c>
       <c r="D6" t="n">
-        <v>16.48936</v>
+        <v>16.54114</v>
       </c>
       <c r="E6" t="n">
-        <v>16.91589</v>
+        <v>16.68693</v>
       </c>
       <c r="F6" t="n">
-        <v>42.68534</v>
+        <v>42.55527</v>
       </c>
       <c r="G6" t="n">
-        <v>0.05222</v>
+        <v>0.05052</v>
       </c>
       <c r="H6" t="n">
-        <v>1.82125</v>
+        <v>1.81726</v>
       </c>
     </row>
     <row r="7">
@@ -585,22 +585,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.67714</v>
+        <v>17.03627</v>
       </c>
       <c r="D7" t="n">
-        <v>16.62876</v>
+        <v>16.14043</v>
       </c>
       <c r="E7" t="n">
-        <v>16.77447</v>
+        <v>16.94054</v>
       </c>
       <c r="F7" t="n">
-        <v>42.74596</v>
+        <v>42.81299</v>
       </c>
       <c r="G7" t="n">
-        <v>0.05127</v>
+        <v>0.04993</v>
       </c>
       <c r="H7" t="n">
-        <v>1.8622</v>
+        <v>1.87467</v>
       </c>
     </row>
     <row r="8">
@@ -610,22 +610,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>16.96869</v>
+        <v>16.81919</v>
       </c>
       <c r="D8" t="n">
-        <v>16.74221</v>
+        <v>16.31395</v>
       </c>
       <c r="E8" t="n">
-        <v>16.82506</v>
+        <v>16.59594</v>
       </c>
       <c r="F8" t="n">
-        <v>43.07741</v>
+        <v>43.25657</v>
       </c>
       <c r="G8" t="n">
-        <v>0.05061</v>
+        <v>0.05121</v>
       </c>
       <c r="H8" t="n">
-        <v>1.84153</v>
+        <v>1.82069</v>
       </c>
     </row>
     <row r="9">
@@ -635,22 +635,22 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>16.95842</v>
+        <v>16.96734</v>
       </c>
       <c r="D9" t="n">
-        <v>16.60329</v>
+        <v>16.57332</v>
       </c>
       <c r="E9" t="n">
-        <v>16.58544</v>
+        <v>16.66453</v>
       </c>
       <c r="F9" t="n">
-        <v>42.25933</v>
+        <v>42.26665</v>
       </c>
       <c r="G9" t="n">
-        <v>0.05115</v>
+        <v>0.05097</v>
       </c>
       <c r="H9" t="n">
-        <v>1.87587</v>
+        <v>1.81833</v>
       </c>
     </row>
     <row r="10">
@@ -660,22 +660,22 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>16.76945</v>
+        <v>16.90301</v>
       </c>
       <c r="D10" t="n">
-        <v>16.6039</v>
+        <v>16.61993</v>
       </c>
       <c r="E10" t="n">
-        <v>16.77349</v>
+        <v>16.90119</v>
       </c>
       <c r="F10" t="n">
-        <v>41.48049</v>
+        <v>42.93646</v>
       </c>
       <c r="G10" t="n">
-        <v>0.05062</v>
+        <v>0.05151</v>
       </c>
       <c r="H10" t="n">
-        <v>1.81902</v>
+        <v>1.80848</v>
       </c>
     </row>
     <row r="11">
@@ -718,26 +718,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pad 2</t>
+          <t>Pad Pos 2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>16.91576</v>
+        <v>17.01327</v>
       </c>
       <c r="D12" t="n">
-        <v>16.69092</v>
+        <v>16.51574</v>
       </c>
       <c r="E12" t="n">
-        <v>16.66535</v>
+        <v>16.71058</v>
       </c>
       <c r="F12" t="n">
-        <v>43.05089</v>
+        <v>43.45668</v>
       </c>
       <c r="G12" t="n">
-        <v>0.05092</v>
+        <v>0.0521</v>
       </c>
       <c r="H12" t="n">
-        <v>1.84467</v>
+        <v>1.82781</v>
       </c>
     </row>
     <row r="13">
@@ -747,22 +747,22 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>17.03488</v>
+        <v>17.01985</v>
       </c>
       <c r="D13" t="n">
-        <v>16.81419</v>
+        <v>16.42496</v>
       </c>
       <c r="E13" t="n">
-        <v>17.00697</v>
+        <v>16.75615</v>
       </c>
       <c r="F13" t="n">
-        <v>41.69411</v>
+        <v>42.55194</v>
       </c>
       <c r="G13" t="n">
-        <v>0.05076</v>
+        <v>0.05004</v>
       </c>
       <c r="H13" t="n">
-        <v>1.84588</v>
+        <v>1.82793</v>
       </c>
     </row>
     <row r="14">
@@ -772,22 +772,22 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>16.91585</v>
+        <v>17.3944</v>
       </c>
       <c r="D14" t="n">
-        <v>16.36109</v>
+        <v>16.80038</v>
       </c>
       <c r="E14" t="n">
-        <v>17.05676</v>
+        <v>16.93149</v>
       </c>
       <c r="F14" t="n">
-        <v>43.23753</v>
+        <v>42.64898</v>
       </c>
       <c r="G14" t="n">
-        <v>0.05005</v>
+        <v>0.05046</v>
       </c>
       <c r="H14" t="n">
-        <v>1.78583</v>
+        <v>1.84247</v>
       </c>
     </row>
     <row r="15">
@@ -797,22 +797,22 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.98073</v>
+        <v>16.96833</v>
       </c>
       <c r="D15" t="n">
-        <v>16.67453</v>
+        <v>16.55936</v>
       </c>
       <c r="E15" t="n">
-        <v>16.78715</v>
+        <v>16.77828</v>
       </c>
       <c r="F15" t="n">
-        <v>42.08607</v>
+        <v>43.2037</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0514</v>
+        <v>0.05137</v>
       </c>
       <c r="H15" t="n">
-        <v>1.84519</v>
+        <v>1.83639</v>
       </c>
     </row>
     <row r="16">
@@ -822,22 +822,22 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>16.94105</v>
+        <v>17.26405</v>
       </c>
       <c r="D16" t="n">
-        <v>16.48614</v>
+        <v>16.65819</v>
       </c>
       <c r="E16" t="n">
-        <v>17.03782</v>
+        <v>16.81578</v>
       </c>
       <c r="F16" t="n">
-        <v>43.24897</v>
+        <v>42.16277</v>
       </c>
       <c r="G16" t="n">
-        <v>0.05032</v>
+        <v>0.05089</v>
       </c>
       <c r="H16" t="n">
-        <v>1.81409</v>
+        <v>1.82961</v>
       </c>
     </row>
     <row r="17">
@@ -847,22 +847,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>16.62507</v>
+        <v>17.27658</v>
       </c>
       <c r="D17" t="n">
-        <v>16.97269</v>
+        <v>16.60145</v>
       </c>
       <c r="E17" t="n">
-        <v>16.83907</v>
+        <v>16.975</v>
       </c>
       <c r="F17" t="n">
-        <v>43.31518</v>
+        <v>43.22728</v>
       </c>
       <c r="G17" t="n">
-        <v>0.05097</v>
+        <v>0.04994</v>
       </c>
       <c r="H17" t="n">
-        <v>1.83394</v>
+        <v>1.80486</v>
       </c>
     </row>
     <row r="18">
@@ -872,22 +872,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>17.15429</v>
+        <v>16.82584</v>
       </c>
       <c r="D18" t="n">
-        <v>16.69204</v>
+        <v>16.44497</v>
       </c>
       <c r="E18" t="n">
-        <v>16.64663</v>
+        <v>16.77324</v>
       </c>
       <c r="F18" t="n">
-        <v>42.22072</v>
+        <v>42.85298</v>
       </c>
       <c r="G18" t="n">
-        <v>0.05162</v>
+        <v>0.05114</v>
       </c>
       <c r="H18" t="n">
-        <v>1.80716</v>
+        <v>1.85109</v>
       </c>
     </row>
     <row r="19">
@@ -897,22 +897,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>16.84201</v>
+        <v>17.21785</v>
       </c>
       <c r="D19" t="n">
-        <v>16.86465</v>
+        <v>16.37156</v>
       </c>
       <c r="E19" t="n">
-        <v>16.9317</v>
+        <v>17.11028</v>
       </c>
       <c r="F19" t="n">
-        <v>43.10889</v>
+        <v>42.57885</v>
       </c>
       <c r="G19" t="n">
-        <v>0.05051</v>
+        <v>0.05171</v>
       </c>
       <c r="H19" t="n">
-        <v>1.83221</v>
+        <v>1.85685</v>
       </c>
     </row>
     <row r="20">
@@ -922,22 +922,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>17.02245</v>
+        <v>16.79627</v>
       </c>
       <c r="D20" t="n">
-        <v>17.06518</v>
+        <v>16.43371</v>
       </c>
       <c r="E20" t="n">
-        <v>16.89911</v>
+        <v>16.72521</v>
       </c>
       <c r="F20" t="n">
-        <v>42.86984</v>
+        <v>42.95835</v>
       </c>
       <c r="G20" t="n">
-        <v>0.05051</v>
+        <v>0.05037</v>
       </c>
       <c r="H20" t="n">
-        <v>1.83658</v>
+        <v>1.85017</v>
       </c>
     </row>
     <row r="21">
@@ -970,20 +970,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SR Pad 1</t>
+          <t>SR Pad Pos 1</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>15.87514</v>
+        <v>16.08329</v>
       </c>
       <c r="D22" t="n">
-        <v>15.63115</v>
+        <v>15.56357</v>
       </c>
       <c r="E22" t="n">
-        <v>16.03974</v>
+        <v>15.81952</v>
       </c>
       <c r="F22" t="n">
-        <v>260.71112</v>
+        <v>255.65231</v>
       </c>
     </row>
     <row r="23">
@@ -993,16 +993,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>15.89434</v>
+        <v>16.29345</v>
       </c>
       <c r="D23" t="n">
-        <v>15.65377</v>
+        <v>15.64793</v>
       </c>
       <c r="E23" t="n">
-        <v>15.727</v>
+        <v>15.69746</v>
       </c>
       <c r="F23" t="n">
-        <v>260.6952</v>
+        <v>256.17011</v>
       </c>
     </row>
     <row r="24">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>15.85951</v>
+        <v>15.86097</v>
       </c>
       <c r="D24" t="n">
-        <v>15.67831</v>
+        <v>15.45123</v>
       </c>
       <c r="E24" t="n">
-        <v>15.92841</v>
+        <v>15.64408</v>
       </c>
       <c r="F24" t="n">
-        <v>257.27256</v>
+        <v>251.91939</v>
       </c>
     </row>
     <row r="25">
@@ -1031,16 +1031,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>15.55463</v>
+        <v>15.75725</v>
       </c>
       <c r="D25" t="n">
-        <v>15.62392</v>
+        <v>15.47842</v>
       </c>
       <c r="E25" t="n">
-        <v>15.74609</v>
+        <v>15.69136</v>
       </c>
       <c r="F25" t="n">
-        <v>257.65745</v>
+        <v>255.7285</v>
       </c>
     </row>
     <row r="26">
@@ -1050,16 +1050,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>15.82608</v>
+        <v>15.93856</v>
       </c>
       <c r="D26" t="n">
-        <v>15.647</v>
+        <v>15.51405</v>
       </c>
       <c r="E26" t="n">
-        <v>15.78028</v>
+        <v>15.7582</v>
       </c>
       <c r="F26" t="n">
-        <v>254.19076</v>
+        <v>256.84013</v>
       </c>
     </row>
     <row r="27">
@@ -1069,16 +1069,16 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>15.69805</v>
+        <v>15.93347</v>
       </c>
       <c r="D27" t="n">
-        <v>15.6441</v>
+        <v>15.61614</v>
       </c>
       <c r="E27" t="n">
-        <v>15.84125</v>
+        <v>15.72912</v>
       </c>
       <c r="F27" t="n">
-        <v>260.40748</v>
+        <v>257.99217</v>
       </c>
     </row>
     <row r="28">
@@ -1088,16 +1088,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>15.80733</v>
+        <v>15.67807</v>
       </c>
       <c r="D28" t="n">
-        <v>15.82871</v>
+        <v>15.53179</v>
       </c>
       <c r="E28" t="n">
-        <v>15.61039</v>
+        <v>15.54267</v>
       </c>
       <c r="F28" t="n">
-        <v>254.44728</v>
+        <v>253.15742</v>
       </c>
     </row>
     <row r="29">
@@ -1107,16 +1107,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>15.69404</v>
+        <v>15.67387</v>
       </c>
       <c r="D29" t="n">
-        <v>15.71486</v>
+        <v>15.536</v>
       </c>
       <c r="E29" t="n">
-        <v>15.97659</v>
+        <v>15.65258</v>
       </c>
       <c r="F29" t="n">
-        <v>258.42967</v>
+        <v>258.00302</v>
       </c>
     </row>
     <row r="30">
@@ -1126,16 +1126,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>15.65264</v>
+        <v>16.0198</v>
       </c>
       <c r="D30" t="n">
-        <v>15.75436</v>
+        <v>15.71348</v>
       </c>
       <c r="E30" t="n">
-        <v>15.65453</v>
+        <v>15.80343</v>
       </c>
       <c r="F30" t="n">
-        <v>254.79944</v>
+        <v>258.97325</v>
       </c>
     </row>
     <row r="31">
@@ -1173,23 +1173,23 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Trace 1</t>
+          <t>Trace Pos 1</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>16.81676</v>
+        <v>16.94632</v>
       </c>
       <c r="D32" t="n">
-        <v>16.19183</v>
+        <v>15.47187</v>
       </c>
       <c r="E32" t="n">
-        <v>16.6793</v>
+        <v>16.53371</v>
       </c>
       <c r="F32" t="n">
-        <v>21.99685</v>
+        <v>21.72512</v>
       </c>
       <c r="G32" t="n">
-        <v>34.9368</v>
+        <v>33.8126</v>
       </c>
     </row>
     <row r="33">
@@ -1199,19 +1199,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>16.974</v>
+        <v>17.19628</v>
       </c>
       <c r="D33" t="n">
-        <v>16.72493</v>
+        <v>15.661</v>
       </c>
       <c r="E33" t="n">
-        <v>16.28366</v>
+        <v>16.6401</v>
       </c>
       <c r="F33" t="n">
-        <v>21.58971</v>
+        <v>21.29034</v>
       </c>
       <c r="G33" t="n">
-        <v>34.60117</v>
+        <v>34.62487</v>
       </c>
     </row>
     <row r="34">
@@ -1221,19 +1221,19 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>16.82083</v>
+        <v>16.78806</v>
       </c>
       <c r="D34" t="n">
-        <v>15.94339</v>
+        <v>15.93061</v>
       </c>
       <c r="E34" t="n">
-        <v>16.42723</v>
+        <v>16.55176</v>
       </c>
       <c r="F34" t="n">
-        <v>21.82685</v>
+        <v>21.93502</v>
       </c>
       <c r="G34" t="n">
-        <v>34.34242</v>
+        <v>34.59314</v>
       </c>
     </row>
     <row r="35">
@@ -1243,19 +1243,19 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>16.77218</v>
+        <v>16.59019</v>
       </c>
       <c r="D35" t="n">
-        <v>16.10258</v>
+        <v>15.93924</v>
       </c>
       <c r="E35" t="n">
-        <v>16.19103</v>
+        <v>16.56728</v>
       </c>
       <c r="F35" t="n">
-        <v>21.85957</v>
+        <v>22.25612</v>
       </c>
       <c r="G35" t="n">
-        <v>34.14718</v>
+        <v>34.67701</v>
       </c>
     </row>
     <row r="36">
@@ -1265,19 +1265,19 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>16.87638</v>
+        <v>17.01209</v>
       </c>
       <c r="D36" t="n">
-        <v>16.04316</v>
+        <v>16.2501</v>
       </c>
       <c r="E36" t="n">
-        <v>16.29898</v>
+        <v>16.30284</v>
       </c>
       <c r="F36" t="n">
-        <v>21.61768</v>
+        <v>21.82145</v>
       </c>
       <c r="G36" t="n">
-        <v>34.05951</v>
+        <v>34.49423</v>
       </c>
     </row>
     <row r="37">
@@ -1287,19 +1287,19 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>16.33334</v>
+        <v>17.07857</v>
       </c>
       <c r="D37" t="n">
-        <v>16.02632</v>
+        <v>16.0001</v>
       </c>
       <c r="E37" t="n">
-        <v>16.29906</v>
+        <v>16.42008</v>
       </c>
       <c r="F37" t="n">
-        <v>21.78502</v>
+        <v>22.03456</v>
       </c>
       <c r="G37" t="n">
-        <v>34.32803</v>
+        <v>34.28177</v>
       </c>
     </row>
     <row r="38">
@@ -1309,19 +1309,19 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>16.94003</v>
+        <v>16.8149</v>
       </c>
       <c r="D38" t="n">
-        <v>16.18252</v>
+        <v>16.24043</v>
       </c>
       <c r="E38" t="n">
-        <v>16.44362</v>
+        <v>16.52516</v>
       </c>
       <c r="F38" t="n">
-        <v>21.91746</v>
+        <v>21.79579</v>
       </c>
       <c r="G38" t="n">
-        <v>34.43245</v>
+        <v>34.95292</v>
       </c>
     </row>
     <row r="39">
@@ -1331,19 +1331,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>16.85044</v>
+        <v>16.67169</v>
       </c>
       <c r="D39" t="n">
-        <v>15.69978</v>
+        <v>16.11422</v>
       </c>
       <c r="E39" t="n">
-        <v>16.53017</v>
+        <v>16.41065</v>
       </c>
       <c r="F39" t="n">
-        <v>22.01695</v>
+        <v>21.68791</v>
       </c>
       <c r="G39" t="n">
-        <v>33.77358</v>
+        <v>33.78112</v>
       </c>
     </row>
     <row r="40">
@@ -1353,45 +1353,30 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>17.08735</v>
+        <v>16.68373</v>
       </c>
       <c r="D40" t="n">
-        <v>16.17314</v>
+        <v>16.20785</v>
       </c>
       <c r="E40" t="n">
-        <v>16.89927</v>
+        <v>16.35625</v>
       </c>
       <c r="F40" t="n">
-        <v>21.74539</v>
+        <v>21.88158</v>
       </c>
       <c r="G40" t="n">
-        <v>35.27789</v>
+        <v>34.94026</v>
       </c>
     </row>
     <row r="41">
       <c r="C41" t="inlineStr">
         <is>
-          <t>Max Stepheight</t>
+          <t>Dimple</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Min Stepheight</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Mean Stepheight</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Width</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Space</t>
+          <t>Bump</t>
         </is>
       </c>
     </row>
@@ -1403,23 +1388,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Trace 2</t>
+          <t>Via Pos 1</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>16.72524</v>
+        <v>0.60638</v>
       </c>
       <c r="D42" t="n">
-        <v>15.88689</v>
-      </c>
-      <c r="E42" t="n">
-        <v>16.5642</v>
-      </c>
-      <c r="F42" t="n">
-        <v>22.06601</v>
-      </c>
-      <c r="G42" t="n">
-        <v>34.08109</v>
+        <v>1.1159</v>
       </c>
     </row>
     <row r="43">
@@ -1429,19 +1405,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>16.57017</v>
+        <v>0.62097</v>
       </c>
       <c r="D43" t="n">
-        <v>16.0264</v>
-      </c>
-      <c r="E43" t="n">
-        <v>16.60828</v>
-      </c>
-      <c r="F43" t="n">
-        <v>22.14729</v>
-      </c>
-      <c r="G43" t="n">
-        <v>34.89907</v>
+        <v>1.10445</v>
       </c>
     </row>
     <row r="44">
@@ -1451,19 +1418,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>16.7447</v>
+        <v>0.607</v>
       </c>
       <c r="D44" t="n">
-        <v>16.00463</v>
-      </c>
-      <c r="E44" t="n">
-        <v>16.45735</v>
-      </c>
-      <c r="F44" t="n">
-        <v>22.21405</v>
-      </c>
-      <c r="G44" t="n">
-        <v>33.44047</v>
+        <v>1.1092</v>
       </c>
     </row>
     <row r="45">
@@ -1473,19 +1431,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>16.58641</v>
+        <v>0.60027</v>
       </c>
       <c r="D45" t="n">
-        <v>15.93598</v>
-      </c>
-      <c r="E45" t="n">
-        <v>16.62508</v>
-      </c>
-      <c r="F45" t="n">
-        <v>21.78425</v>
-      </c>
-      <c r="G45" t="n">
-        <v>34.14886</v>
+        <v>1.12484</v>
       </c>
     </row>
     <row r="46">
@@ -1495,19 +1444,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>16.65819</v>
+        <v>0.61158</v>
       </c>
       <c r="D46" t="n">
-        <v>16.12413</v>
-      </c>
-      <c r="E46" t="n">
-        <v>15.94359</v>
-      </c>
-      <c r="F46" t="n">
-        <v>22.19877</v>
-      </c>
-      <c r="G46" t="n">
-        <v>34.45426</v>
+        <v>1.13483</v>
       </c>
     </row>
     <row r="47">
@@ -1517,19 +1457,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>16.47597</v>
+        <v>0.5993000000000001</v>
       </c>
       <c r="D47" t="n">
-        <v>16.45546</v>
-      </c>
-      <c r="E47" t="n">
-        <v>16.19604</v>
-      </c>
-      <c r="F47" t="n">
-        <v>21.38719</v>
-      </c>
-      <c r="G47" t="n">
-        <v>34.45385</v>
+        <v>1.12382</v>
       </c>
     </row>
     <row r="48">
@@ -1539,19 +1470,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>16.99365</v>
+        <v>0.60121</v>
       </c>
       <c r="D48" t="n">
-        <v>16.18237</v>
-      </c>
-      <c r="E48" t="n">
-        <v>16.38619</v>
-      </c>
-      <c r="F48" t="n">
-        <v>21.97577</v>
-      </c>
-      <c r="G48" t="n">
-        <v>34.15721</v>
+        <v>1.13317</v>
       </c>
     </row>
     <row r="49">
@@ -1561,19 +1483,10 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>16.66453</v>
+        <v>0.62391</v>
       </c>
       <c r="D49" t="n">
-        <v>15.90031</v>
-      </c>
-      <c r="E49" t="n">
-        <v>16.51356</v>
-      </c>
-      <c r="F49" t="n">
-        <v>21.71896</v>
-      </c>
-      <c r="G49" t="n">
-        <v>34.41326</v>
+        <v>1.11623</v>
       </c>
     </row>
     <row r="50">
@@ -1583,30 +1496,31 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>16.72127</v>
+        <v>0.62434</v>
       </c>
       <c r="D50" t="n">
-        <v>16.18591</v>
-      </c>
-      <c r="E50" t="n">
-        <v>16.5612</v>
-      </c>
-      <c r="F50" t="n">
-        <v>22.14886</v>
-      </c>
-      <c r="G50" t="n">
-        <v>33.95915</v>
+        <v>1.10286</v>
       </c>
     </row>
     <row r="51">
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dimple</t>
+          <t>Max Stepheight</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Bump</t>
+          <t>Min Stepheight</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Mean Stepheight</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Radius</t>
         </is>
       </c>
     </row>
@@ -1618,14 +1532,20 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>via 1</t>
+          <t>Landing Pad 1</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.61494</v>
+        <v>16.94853</v>
       </c>
       <c r="D52" t="n">
-        <v>1.10776</v>
+        <v>16.71777</v>
+      </c>
+      <c r="E52" t="n">
+        <v>16.8082</v>
+      </c>
+      <c r="F52" t="n">
+        <v>43.00742</v>
       </c>
     </row>
     <row r="53">
@@ -1635,10 +1555,16 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.60766</v>
+        <v>16.83096</v>
       </c>
       <c r="D53" t="n">
-        <v>1.13815</v>
+        <v>16.49043</v>
+      </c>
+      <c r="E53" t="n">
+        <v>16.81942</v>
+      </c>
+      <c r="F53" t="n">
+        <v>42.56048</v>
       </c>
     </row>
     <row r="54">
@@ -1648,10 +1574,16 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0.6252</v>
+        <v>16.9673</v>
       </c>
       <c r="D54" t="n">
-        <v>1.117</v>
+        <v>16.62944</v>
+      </c>
+      <c r="E54" t="n">
+        <v>16.76168</v>
+      </c>
+      <c r="F54" t="n">
+        <v>43.42931</v>
       </c>
     </row>
     <row r="55">
@@ -1661,10 +1593,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0.6151799999999999</v>
+        <v>17.09375</v>
       </c>
       <c r="D55" t="n">
-        <v>1.10167</v>
+        <v>16.70927</v>
+      </c>
+      <c r="E55" t="n">
+        <v>16.94233</v>
+      </c>
+      <c r="F55" t="n">
+        <v>43.76185</v>
       </c>
     </row>
     <row r="56">
@@ -1674,10 +1612,16 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0.60931</v>
+        <v>16.9199</v>
       </c>
       <c r="D56" t="n">
-        <v>1.11446</v>
+        <v>16.64439</v>
+      </c>
+      <c r="E56" t="n">
+        <v>16.73007</v>
+      </c>
+      <c r="F56" t="n">
+        <v>42.38526</v>
       </c>
     </row>
     <row r="57">
@@ -1687,10 +1631,16 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0.60048</v>
+        <v>17.07879</v>
       </c>
       <c r="D57" t="n">
-        <v>1.11707</v>
+        <v>16.5468</v>
+      </c>
+      <c r="E57" t="n">
+        <v>16.65783</v>
+      </c>
+      <c r="F57" t="n">
+        <v>42.84158</v>
       </c>
     </row>
     <row r="58">
@@ -1700,10 +1650,16 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.62871</v>
+        <v>17.14373</v>
       </c>
       <c r="D58" t="n">
-        <v>1.13565</v>
+        <v>16.7821</v>
+      </c>
+      <c r="E58" t="n">
+        <v>16.97756</v>
+      </c>
+      <c r="F58" t="n">
+        <v>43.09494</v>
       </c>
     </row>
     <row r="59">
@@ -1713,10 +1669,16 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.61092</v>
+        <v>17.06658</v>
       </c>
       <c r="D59" t="n">
-        <v>1.117</v>
+        <v>16.43519</v>
+      </c>
+      <c r="E59" t="n">
+        <v>16.72612</v>
+      </c>
+      <c r="F59" t="n">
+        <v>42.69009</v>
       </c>
     </row>
     <row r="60">
@@ -1726,144 +1688,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.6055199999999999</v>
+        <v>17.16977</v>
       </c>
       <c r="D60" t="n">
-        <v>1.12595</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Dimple</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Bump</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Unit 7</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>via 2</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>0.59853</v>
-      </c>
-      <c r="D62" t="n">
-        <v>1.12537</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Unit 8</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>0.61703</v>
-      </c>
-      <c r="D63" t="n">
-        <v>1.13153</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Unit 9</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>0.61644</v>
-      </c>
-      <c r="D64" t="n">
-        <v>1.12224</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Unit 4</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>0.6078</v>
-      </c>
-      <c r="D65" t="n">
-        <v>1.11732</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Unit 5</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>0.62778</v>
-      </c>
-      <c r="D66" t="n">
-        <v>1.10426</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Unit 6</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>0.61067</v>
-      </c>
-      <c r="D67" t="n">
-        <v>1.11809</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Unit 1</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>0.6244499999999999</v>
-      </c>
-      <c r="D68" t="n">
-        <v>1.11351</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Unit 2</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>0.61727</v>
-      </c>
-      <c r="D69" t="n">
-        <v>1.13214</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Unit 3</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>0.59924</v>
-      </c>
-      <c r="D70" t="n">
-        <v>1.10297</v>
+        <v>16.66244</v>
+      </c>
+      <c r="E60" t="n">
+        <v>16.70225</v>
+      </c>
+      <c r="F60" t="n">
+        <v>43.19353</v>
       </c>
     </row>
   </sheetData>

</xml_diff>